<commit_message>
add: Plano de Garantia de qualidade e versão dos documentos
fix: checklists nomes e formulas
</commit_message>
<xml_diff>
--- a/CheckLists de autoria/Checklist_Auditoria_Vazio.xlsx
+++ b/CheckLists de autoria/Checklist_Auditoria_Vazio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PlanoGarantiaQualidade\CheckLists de autoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AFDD25A-1673-4715-9509-3FE6A7DED6C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D60C733-D65F-4A54-9652-BFAE808F1CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist - Auditoria" sheetId="1" r:id="rId1"/>
@@ -91,9 +91,6 @@
     <t>Auditor de QA:</t>
   </si>
   <si>
-    <t>Gustavo, André Gritten, Eduardo Blaszczak, Mateus</t>
-  </si>
-  <si>
     <t>Data da auditoria:</t>
   </si>
   <si>
@@ -251,6 +248,9 @@
   </si>
   <si>
     <t>Relatório de Teste de Usabilidade do Sistema Web - iFood</t>
+  </si>
+  <si>
+    <t>Gustavo Giacoia, André Gritten, Eduardo Blasczak, Mateus dos Santos</t>
   </si>
 </sst>
 </file>
@@ -507,27 +507,27 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -832,18 +832,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
     </row>
     <row r="2" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -878,25 +878,25 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
+      <c r="A3" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
     </row>
     <row r="4" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="5"/>
@@ -915,7 +915,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="5"/>
@@ -934,7 +934,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="5"/>
@@ -953,7 +953,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="5"/>
@@ -972,7 +972,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="5"/>
@@ -987,25 +987,25 @@
       <c r="J8" s="4"/>
     </row>
     <row r="9" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="37" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="37"/>
+      <c r="A9" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
     </row>
     <row r="10" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="5"/>
@@ -1024,7 +1024,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="5"/>
@@ -1043,7 +1043,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
@@ -1062,7 +1062,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="5"/>
@@ -1081,7 +1081,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="5"/>
@@ -1096,25 +1096,25 @@
       <c r="J14" s="4"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="37" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="37"/>
+      <c r="A15" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
+      <c r="H15" s="29"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>11</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
@@ -1133,7 +1133,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="5"/>
@@ -1152,7 +1152,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="5"/>
@@ -1171,7 +1171,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="5"/>
@@ -1187,7 +1187,7 @@
     </row>
     <row r="20" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1204,7 +1204,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="5"/>
@@ -1223,7 +1223,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="5"/>
@@ -1239,7 +1239,7 @@
     </row>
     <row r="23" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1256,7 +1256,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="5"/>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="25" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="5"/>
@@ -1288,7 +1288,7 @@
     </row>
     <row r="26" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1305,7 +1305,7 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C27" s="27"/>
       <c r="D27" s="24"/>
@@ -1321,7 +1321,7 @@
         <v>20</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="5"/>
@@ -1391,85 +1391,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
+      <c r="B4" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
+      <c r="B5" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="35">
+        <v>15</v>
+      </c>
+      <c r="B6" s="33">
         <v>46269</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-      <c r="E7" s="29"/>
+        <v>16</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="8">
         <f>COUNTA('Checklist - Auditoria'!$B$3:$B$28)</f>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="8">
         <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Conforme")</f>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="8">
         <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Não Conforme")</f>
@@ -1496,7 +1496,7 @@
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="8">
         <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Não se Aplica")</f>
@@ -1505,7 +1505,7 @@
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="8">
         <f>COUNTIFS('Checklist - Auditoria'!$C$3:$C$28,"Não Conforme",'Checklist - Auditoria'!$J$3:$J$28,"&lt;&gt;Resolvida")</f>
@@ -1513,62 +1513,62 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="30" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="30"/>
+      <c r="A16" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="35"/>
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="31">
+      <c r="A17" s="36">
         <f>IFERROR(B11/(B10-B13),0)</f>
         <v>0</v>
       </c>
-      <c r="B17" s="31"/>
+      <c r="B17" s="36"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="32"/>
+      <c r="A19" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="37"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>29</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>31</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26" s="14">
         <v>90</v>
@@ -1580,7 +1580,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B27" s="14">
         <v>60</v>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" s="14">
         <v>30</v>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="18">
@@ -1658,30 +1658,25 @@
       <c r="G34" s="26"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="28"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="28"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="28"/>
+      <c r="A38" s="34"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="B7:E7"/>
@@ -1689,6 +1684,11 @@
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1696,20 +1696,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1907,14 +1907,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D39D842-B01B-4CD0-AE66-42EBDFD06EF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F57FCCD9-0F54-408C-A072-F3A2C41297DF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1926,6 +1918,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6D39D842-B01B-4CD0-AE66-42EBDFD06EF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>